<commit_message>
Regenerated 837 converted files
</commit_message>
<xml_diff>
--- a/converted_files/837/837I-all-fields.xlsx
+++ b/converted_files/837/837I-all-fields.xlsx
@@ -1872,7 +1872,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>6a04cc5b1ef26d534baf3f2b</t>
+          <t>6a0614def8d6a2fc74348d75</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="J2" s="1" t="n">
-        <v>89.93</v>
+        <v>259.96</v>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
@@ -1943,7 +1943,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="P2"/>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>NPI</t>
@@ -2257,7 +2261,9 @@
           <t>01</t>
         </is>
       </c>
-      <c r="CT2"/>
+      <c r="CT2" s="1" t="n">
+        <v>123.0</v>
+      </c>
       <c r="CU2" s="3" t="inlineStr">
         <is>
           <t>1</t>
@@ -3073,10 +3079,22 @@
       <c r="KY2" s="4" t="n">
         <v>43596.0</v>
       </c>
-      <c r="KZ2"/>
-      <c r="LA2"/>
-      <c r="LB2"/>
-      <c r="LC2"/>
+      <c r="KZ2" s="3" t="inlineStr">
+        <is>
+          <t>Repriced</t>
+        </is>
+      </c>
+      <c r="LA2" s="3" t="inlineStr">
+        <is>
+          <t>AdjRepriced</t>
+        </is>
+      </c>
+      <c r="LB2" s="1" t="n">
+        <v>15.0</v>
+      </c>
+      <c r="LC2" s="1" t="n">
+        <v>22.0</v>
+      </c>
       <c r="LD2" s="3" t="inlineStr">
         <is>
           <t>state regulation 123 was applied during the pricing of this claim</t>
@@ -3092,7 +3110,7 @@
       </c>
       <c r="LG2" s="3" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>GRAM</t>
         </is>
       </c>
       <c r="LH2" s="3" t="inlineStr">
@@ -3107,7 +3125,7 @@
       </c>
       <c r="LJ2" s="3" t="inlineStr">
         <is>
-          <t>BM</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="LK2" s="3" t="inlineStr">
@@ -3221,7 +3239,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>6a04cc5b1ef26d534baf3f2b</t>
+          <t>6a0614def8d6a2fc74348d75</t>
         </is>
       </c>
       <c r="B3"/>
@@ -3609,12 +3627,12 @@
       </c>
       <c r="LI3" s="3" t="inlineStr">
         <is>
-          <t>ZZ</t>
+          <t>08</t>
         </is>
       </c>
       <c r="LJ3" s="3" t="inlineStr">
         <is>
-          <t>BC</t>
+          <t>EL</t>
         </is>
       </c>
       <c r="LK3" s="3" t="inlineStr">

</xml_diff>